<commit_message>
feat: changed headbar for Cennik.js feat: added style for table in Cennik.js
</commit_message>
<xml_diff>
--- a/backend/data/cennik.xlsx
+++ b/backend/data/cennik.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\StronaMonikaReact\config\node\backend\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\StronaMonika\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7DF384A-FCEB-4E4C-9EBA-E8CA72448F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B5F11BC-D840-4BE1-91B0-9B1912239819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>Pedicure</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="109">
   <si>
     <t>NAZWA</t>
   </si>
@@ -50,32 +47,329 @@
     <t>CENA</t>
   </si>
   <si>
-    <t>abcdef</t>
-  </si>
-  <si>
-    <t>Manicure</t>
-  </si>
-  <si>
-    <t>eeeee</t>
-  </si>
-  <si>
-    <t>Botoks</t>
-  </si>
-  <si>
-    <t>Zabieg et</t>
-  </si>
-  <si>
-    <t>Oczyszczanie</t>
-  </si>
-  <si>
-    <t>Opis</t>
+    <t>Oczyszczanie manualne</t>
+  </si>
+  <si>
+    <t>Ręczne usuwanie zaskórników i niedoskonałości skóry.</t>
+  </si>
+  <si>
+    <t>Oczyszczanie wodorowe</t>
+  </si>
+  <si>
+    <t>Dogłębne oczyszczanie skóry aktywnym wodorem.</t>
+  </si>
+  <si>
+    <t>Peeling kawitacyjny</t>
+  </si>
+  <si>
+    <t>Ultradźwiękowe złuszczanie martwego naskórka.</t>
+  </si>
+  <si>
+    <t>Mikrodermabrazja diamentowa</t>
+  </si>
+  <si>
+    <t>Mechaniczne wygładzenie i odnowa skóry.</t>
+  </si>
+  <si>
+    <t>Infuzja tlenowa</t>
+  </si>
+  <si>
+    <t>Dotlenienie i nawilżenie skóry pod ciśnieniem.</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 1</t>
+  </si>
+  <si>
+    <t>Profesjonalny zabieg poprawiający kondycję skóry.</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 2</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 3</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 4</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 5</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 6</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 7</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 8</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 9</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 10</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 11</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 12</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 13</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 14</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 15</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 16</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 17</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 18</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 19</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 20</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 21</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 22</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 23</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 24</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 25</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 26</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 27</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 28</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 29</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 30</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 31</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 32</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 33</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 34</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 35</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 36</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 37</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 38</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 39</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 40</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 41</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 42</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 43</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 44</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 45</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 46</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 47</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 48</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 49</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 50</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 51</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 52</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 53</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 54</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 55</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 56</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 57</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 58</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 59</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 60</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 61</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 62</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 63</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 64</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 65</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 66</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 67</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 68</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 69</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 70</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 71</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 72</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 73</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 74</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 75</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 76</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 77</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 78</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 79</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 80</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 81</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 82</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 83</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 84</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 85</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 86</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 87</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 88</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 89</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 90</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 91</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 92</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 93</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 94</t>
+  </si>
+  <si>
+    <t>Zabieg pielęgnacyjny 95</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -105,7 +399,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -441,62 +736,1118 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED3D7DE2-9127-49D9-96AA-B2504799E15F}">
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C101"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>200</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="C3" s="1">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C4">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="C4" s="1">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C5">
-        <v>500</v>
+      <c r="C5" s="1">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="1">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="1">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="1">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="1">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="1">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="1">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="1">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="1">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="1">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="1">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="1">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="1">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" s="1">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="1">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" s="1">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" s="1">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="1">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" s="1">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" s="1">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" s="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C31" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" s="1">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C33" s="1">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="1">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="1">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" s="1">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" s="1">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" s="1">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C39" s="1">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C40" s="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C41" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C42" s="1">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C43" s="1">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C44" s="1">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C45" s="1">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C46" s="1">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C47" s="1">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C48" s="1">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C49" s="1">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C50" s="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C51" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C52" s="1">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C53" s="1">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C54" s="1">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C55" s="1">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C56" s="1">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C57" s="1">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C58" s="1">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C59" s="1">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C60" s="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C61" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C62" s="1">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C63" s="1">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C64" s="1">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C65" s="1">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C66" s="1">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C67" s="1">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C68" s="1">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C69" s="1">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C70" s="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C71" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C72" s="1">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C73" s="1">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C74" s="1">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C75" s="1">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C76" s="1">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C77" s="1">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C78" s="1">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="A79" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C79" s="1">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="A80" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C80" s="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3">
+      <c r="A81" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C81" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3">
+      <c r="A82" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C82" s="1">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3">
+      <c r="A83" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C83" s="1">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3">
+      <c r="A84" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C84" s="1">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3">
+      <c r="A85" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C85" s="1">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3">
+      <c r="A86" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C86" s="1">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3">
+      <c r="A87" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C87" s="1">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3">
+      <c r="A88" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C88" s="1">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3">
+      <c r="A89" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C89" s="1">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3">
+      <c r="A90" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C90" s="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3">
+      <c r="A91" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C91" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3">
+      <c r="A92" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C92" s="1">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3">
+      <c r="A93" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C93" s="1">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3">
+      <c r="A94" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C94" s="1">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3">
+      <c r="A95" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C95" s="1">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3">
+      <c r="A96" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C96" s="1">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3">
+      <c r="A97" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C97" s="1">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3">
+      <c r="A98" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C98" s="1">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3">
+      <c r="A99" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C99" s="1">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3">
+      <c r="A100" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C100" s="1">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3">
+      <c r="A101" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C101" s="1">
+        <v>250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
wip: added pickedTreatmentLoad.js which loads content from word files.
</commit_message>
<xml_diff>
--- a/backend/data/cennik.xlsx
+++ b/backend/data/cennik.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\StronaMonikaJS\backend\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\StronaMonika\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F829CCCC-D67C-4FE3-BF2E-3BAA7CDBFDB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC225CB-FFAA-4FF1-BC29-0447F4E23759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="151">
   <si>
     <t>OPIS</t>
   </si>
@@ -47,9 +47,6 @@
     <t>Pierwszy zabieg</t>
   </si>
   <si>
-    <t>Makjiaż permanentny brwi - Odświeżenie</t>
-  </si>
-  <si>
     <t>Makijaż permanentny brwi pudrowe</t>
   </si>
   <si>
@@ -80,12 +77,6 @@
     <t>???????</t>
   </si>
   <si>
-    <t>Do 1,5 roku od wykonania pierwszego zabiegu</t>
-  </si>
-  <si>
-    <t>Od 1,5 roku do 2 lat od wykonania pierwszego zabiegu</t>
-  </si>
-  <si>
     <t>Do 2 lat od wykonania pierwszego zabiegu</t>
   </si>
   <si>
@@ -173,12 +164,6 @@
     <t>Depilacja tłowiu</t>
   </si>
   <si>
-    <t>Depilacja woskiem karku</t>
-  </si>
-  <si>
-    <t>Depilacja woskiem połowy pleców z karkiem/klatką piersiową</t>
-  </si>
-  <si>
     <t>Depilacja woskiem całych pleców</t>
   </si>
   <si>
@@ -264,6 +249,246 @@
   </si>
   <si>
     <t>CZASZABIEGU</t>
+  </si>
+  <si>
+    <t>Manicure Biologiczny Tradycyjny</t>
+  </si>
+  <si>
+    <t>50 min</t>
+  </si>
+  <si>
+    <t>65 min</t>
+  </si>
+  <si>
+    <t>Bez Malowania</t>
+  </si>
+  <si>
+    <t>Z malowaniem jeden kolor/odżywka</t>
+  </si>
+  <si>
+    <t>Z malowaniem french</t>
+  </si>
+  <si>
+    <t>Manicure Japoński</t>
+  </si>
+  <si>
+    <t>Regeneracja Płytki Paznokciowej</t>
+  </si>
+  <si>
+    <t>Depilacja Woskiem Karku</t>
+  </si>
+  <si>
+    <t>Depilacja Woskiem Połowy pleców z karkiem/klatką piersiową</t>
+  </si>
+  <si>
+    <t>Manicure Hybrydowy</t>
+  </si>
+  <si>
+    <t>90 - 100 min</t>
+  </si>
+  <si>
+    <t>Baza Hybrydowa</t>
+  </si>
+  <si>
+    <t>Z malowaniem na jeden kolor</t>
+  </si>
+  <si>
+    <t>Z Malowaniem French/Babyboomer</t>
+  </si>
+  <si>
+    <t>Ściaganie Hybrydy</t>
+  </si>
+  <si>
+    <t>30 - 40 min</t>
+  </si>
+  <si>
+    <t>Wykonanej w innym salonie przy założeniu nowej stylizacji w Salonie Obsession</t>
+  </si>
+  <si>
+    <t>Wykonanej w innym salonie bez założenia nowej hybrydy</t>
+  </si>
+  <si>
+    <t>Przedłużanie Jednego Paznokcia</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -</t>
+  </si>
+  <si>
+    <t>Pedicure Frezarkowy (Opracowanie Paznokcji i Pięt)</t>
+  </si>
+  <si>
+    <t>Z Malowaniem Na Jeden Kolor/Odżywka</t>
+  </si>
+  <si>
+    <t>Z Malowaniem French</t>
+  </si>
+  <si>
+    <t>Pedicure Hybrydowy (Opracowanie Paznokci i Pięt)</t>
+  </si>
+  <si>
+    <t>100 min</t>
+  </si>
+  <si>
+    <t>Z Malowaniem Na Jeden Kolor</t>
+  </si>
+  <si>
+    <t>Pielęgnacja Płytki Paznokciowej Stóp (bez opracowania pięt)</t>
+  </si>
+  <si>
+    <t>Hybryda Stóp (Bez Opracowania Pięt)</t>
+  </si>
+  <si>
+    <t>Pielęgnacja Pięt</t>
+  </si>
+  <si>
+    <t>30 - 60 min</t>
+  </si>
+  <si>
+    <t>Przy Użyciu Omegi i Frezarki</t>
+  </si>
+  <si>
+    <t>Oczyszczanie Manualne Twarzy</t>
+  </si>
+  <si>
+    <t>Z Maską w Kremie</t>
+  </si>
+  <si>
+    <t>Z Dodatkowym Peelingiem Chemicznym</t>
+  </si>
+  <si>
+    <t>+ 100</t>
+  </si>
+  <si>
+    <t>Peeling Kawitacyjny (Twarz, Szyja, Dekolt)</t>
+  </si>
+  <si>
+    <t>45 min</t>
+  </si>
+  <si>
+    <t>55 min</t>
+  </si>
+  <si>
+    <t>+ 20 min</t>
+  </si>
+  <si>
+    <t>Z Ampułką i Maską Algową</t>
+  </si>
+  <si>
+    <t>Z Dodatkowym Masażem</t>
+  </si>
+  <si>
+    <t>+ 20</t>
+  </si>
+  <si>
+    <t>Mikrodermabrazja Diamentowa z Maską w Kremie</t>
+  </si>
+  <si>
+    <t>40 min</t>
+  </si>
+  <si>
+    <t>+ 15 min</t>
+  </si>
+  <si>
+    <t>Twarz</t>
+  </si>
+  <si>
+    <t>Twarz z Szyją</t>
+  </si>
+  <si>
+    <t>Twarzy, Szyja i Dekolt</t>
+  </si>
+  <si>
+    <t>+ 30</t>
+  </si>
+  <si>
+    <t>Maska Algowa z Ampułką</t>
+  </si>
+  <si>
+    <t>Dodatkowo Do Zabiegu</t>
+  </si>
+  <si>
+    <t>+ 40</t>
+  </si>
+  <si>
+    <t>Peelingi Chemiczne</t>
+  </si>
+  <si>
+    <t>45 - 60 min</t>
+  </si>
+  <si>
+    <t>RETIX C (Twarz, Szyja i Dekolt)</t>
+  </si>
+  <si>
+    <t>RETIX C EYE (Oczy)</t>
+  </si>
+  <si>
+    <t>Kwasy RETIX C (Twarz, Szyja lub Dekolt)</t>
+  </si>
+  <si>
+    <t>AQUA PEEL (Twarz, Szyja, Dekolt)</t>
+  </si>
+  <si>
+    <t>180 - 300</t>
+  </si>
+  <si>
+    <t>LIFT PEEL (Twarz, Szyja, Dekolt)</t>
+  </si>
+  <si>
+    <t>RETI PEEL (Twarz, Szyja, Dekolt)</t>
+  </si>
+  <si>
+    <t>DEPI GEN (Twarz, Szyja, Dekolt)</t>
+  </si>
+  <si>
+    <t>ASIATIC PEEL (Twarz, Szyja, Dekolt)</t>
+  </si>
+  <si>
+    <t>Zabieg Nanoigły (Zabieg na Przebarwienia, Blizny, Zmarszczki, Rozszerzone Pory)</t>
+  </si>
+  <si>
+    <t>Z Jedną Ampułką Nanoigieł</t>
+  </si>
+  <si>
+    <t>Z Dwiema Ampułkami Nanoigieł</t>
+  </si>
+  <si>
+    <t>PqAge (Twarz i Szyja)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DERMAPEN </t>
+  </si>
+  <si>
+    <t>DERMAPEN + PqAge</t>
+  </si>
+  <si>
+    <t>Oczy</t>
+  </si>
+  <si>
+    <t>Twarz/Szyja/Dekolt</t>
+  </si>
+  <si>
+    <t>Twarz + Oczy</t>
+  </si>
+  <si>
+    <t>Twarz + Oczy + Szyja</t>
+  </si>
+  <si>
+    <t>Twarz + Oczy + Szyja + Dekolt</t>
+  </si>
+  <si>
+    <t>DERMAPEN + Peeling Chemiczny</t>
+  </si>
+  <si>
+    <t>Twarz + Szyja</t>
+  </si>
+  <si>
+    <t>Twarz + Szyja + Dekolt</t>
+  </si>
+  <si>
+    <t>Odświeżenie do 1,5 roku od wykonania pierwszego zabiegu</t>
+  </si>
+  <si>
+    <t>Odświeżenie od 1,5 roku do 2 lat od wykonania pierwszego zabiegu</t>
   </si>
 </sst>
 </file>
@@ -300,8 +525,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -636,19 +862,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED3D7DE2-9127-49D9-96AA-B2504799E15F}">
-  <dimension ref="A1:D43"/>
-  <sheetFormatPr defaultColWidth="32" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D101"/>
+  <sheetFormatPr defaultColWidth="32" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.77734375" customWidth="1"/>
-    <col min="4" max="4" width="18.109375" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -657,12 +883,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
         <v>2</v>
@@ -671,40 +897,40 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>149</v>
       </c>
       <c r="D3">
         <v>500</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>150</v>
       </c>
       <c r="D4">
         <v>750</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
         <v>2</v>
@@ -713,536 +939,1348 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D6">
         <v>600</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D7">
         <v>800</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D8">
         <v>700</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>9</v>
       </c>
-      <c r="B9" t="s">
-        <v>10</v>
-      </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D9">
         <v>900</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D10">
         <v>500</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D11">
         <v>500</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D12">
         <v>700</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D13">
         <v>300</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" t="s">
         <v>20</v>
-      </c>
-      <c r="B14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" t="s">
-        <v>23</v>
       </c>
       <c r="D14">
         <v>400</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D15">
         <v>200</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D16">
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C17" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D17">
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C18" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D18">
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C19" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D19">
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C20" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D20">
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" t="s">
         <v>31</v>
-      </c>
-      <c r="B21" t="s">
-        <v>25</v>
-      </c>
-      <c r="C21" t="s">
-        <v>34</v>
       </c>
       <c r="D21">
         <v>115</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C22" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D22">
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C23" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D23">
         <v>60</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B24" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C24" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D24">
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C25" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D25">
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B26" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C26" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D26">
         <v>75</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" t="s">
+        <v>22</v>
+      </c>
+      <c r="C27" t="s">
         <v>40</v>
-      </c>
-      <c r="B27" t="s">
-        <v>25</v>
-      </c>
-      <c r="C27" t="s">
-        <v>43</v>
       </c>
       <c r="D27">
         <v>120</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B28" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C28" t="s">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="D28">
         <v>40</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B29" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C29" t="s">
-        <v>46</v>
+        <v>80</v>
       </c>
       <c r="D29">
         <v>70</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B30" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C30" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D30">
         <v>100</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C31" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D31">
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B32" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C32" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D32">
         <v>120</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B33" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C33" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D33">
         <v>170</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C34" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D34">
         <v>200</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C35" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D35">
         <v>150</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>44</v>
+      </c>
+      <c r="B36" t="s">
+        <v>53</v>
+      </c>
+      <c r="C36" t="s">
         <v>49</v>
-      </c>
-      <c r="B36" t="s">
-        <v>58</v>
-      </c>
-      <c r="C36" t="s">
-        <v>54</v>
       </c>
       <c r="D36">
         <v>60</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B37" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C37" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D37">
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B38" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C38" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D38">
         <v>55</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B39" t="s">
+        <v>53</v>
+      </c>
+      <c r="C39" t="s">
         <v>58</v>
-      </c>
-      <c r="C39" t="s">
-        <v>63</v>
       </c>
       <c r="D39">
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>54</v>
+      </c>
+      <c r="B40" t="s">
+        <v>52</v>
+      </c>
+      <c r="C40" t="s">
         <v>59</v>
-      </c>
-      <c r="B40" t="s">
-        <v>57</v>
-      </c>
-      <c r="C40" t="s">
-        <v>64</v>
       </c>
       <c r="D40">
         <v>145</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B41" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C41" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D41">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B42" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C42" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D42">
         <v>145</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B43" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C43" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D43">
         <v>270</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>71</v>
+      </c>
+      <c r="B44" t="s">
+        <v>72</v>
+      </c>
+      <c r="C44" t="s">
+        <v>74</v>
+      </c>
+      <c r="D44">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>71</v>
+      </c>
+      <c r="B45" t="s">
+        <v>51</v>
+      </c>
+      <c r="C45" t="s">
+        <v>75</v>
+      </c>
+      <c r="D45">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46" t="s">
+        <v>73</v>
+      </c>
+      <c r="C46" t="s">
+        <v>76</v>
+      </c>
+      <c r="D46">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>77</v>
+      </c>
+      <c r="B47" t="s">
+        <v>51</v>
+      </c>
+      <c r="C47" t="s">
+        <v>78</v>
+      </c>
+      <c r="D47">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>81</v>
+      </c>
+      <c r="B48" t="s">
+        <v>51</v>
+      </c>
+      <c r="C48" t="s">
+        <v>83</v>
+      </c>
+      <c r="D48">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>81</v>
+      </c>
+      <c r="B49" t="s">
+        <v>82</v>
+      </c>
+      <c r="C49" t="s">
+        <v>84</v>
+      </c>
+      <c r="D49">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>81</v>
+      </c>
+      <c r="B50" t="s">
+        <v>82</v>
+      </c>
+      <c r="C50" t="s">
+        <v>85</v>
+      </c>
+      <c r="D50">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>86</v>
+      </c>
+      <c r="B51" t="s">
+        <v>55</v>
+      </c>
+      <c r="C51" t="s">
+        <v>88</v>
+      </c>
+      <c r="D51">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>86</v>
+      </c>
+      <c r="B52" t="s">
+        <v>87</v>
+      </c>
+      <c r="C52" t="s">
+        <v>89</v>
+      </c>
+      <c r="D52">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>90</v>
+      </c>
+      <c r="B53" t="s">
+        <v>53</v>
+      </c>
+      <c r="C53" t="s">
+        <v>91</v>
+      </c>
+      <c r="D53">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>92</v>
+      </c>
+      <c r="B54" t="s">
+        <v>64</v>
+      </c>
+      <c r="C54" t="s">
+        <v>74</v>
+      </c>
+      <c r="D54">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>92</v>
+      </c>
+      <c r="B55" t="s">
+        <v>16</v>
+      </c>
+      <c r="C55" t="s">
+        <v>93</v>
+      </c>
+      <c r="D55">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>92</v>
+      </c>
+      <c r="B56" t="s">
+        <v>10</v>
+      </c>
+      <c r="C56" t="s">
+        <v>94</v>
+      </c>
+      <c r="D56">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>95</v>
+      </c>
+      <c r="B57" t="s">
+        <v>10</v>
+      </c>
+      <c r="C57" t="s">
+        <v>83</v>
+      </c>
+      <c r="D57">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>95</v>
+      </c>
+      <c r="B58" t="s">
+        <v>96</v>
+      </c>
+      <c r="C58" t="s">
+        <v>97</v>
+      </c>
+      <c r="D58">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>95</v>
+      </c>
+      <c r="B59" t="s">
+        <v>96</v>
+      </c>
+      <c r="C59" t="s">
+        <v>94</v>
+      </c>
+      <c r="D59">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>98</v>
+      </c>
+      <c r="B60" t="s">
+        <v>72</v>
+      </c>
+      <c r="C60" t="s">
+        <v>74</v>
+      </c>
+      <c r="D60">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>98</v>
+      </c>
+      <c r="B61" t="s">
+        <v>51</v>
+      </c>
+      <c r="C61" t="s">
+        <v>93</v>
+      </c>
+      <c r="D61">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>98</v>
+      </c>
+      <c r="B62" t="s">
+        <v>52</v>
+      </c>
+      <c r="C62" t="s">
+        <v>94</v>
+      </c>
+      <c r="D62">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>99</v>
+      </c>
+      <c r="B63" t="s">
+        <v>51</v>
+      </c>
+      <c r="C63" t="s">
+        <v>83</v>
+      </c>
+      <c r="D63">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>99</v>
+      </c>
+      <c r="B64" t="s">
+        <v>64</v>
+      </c>
+      <c r="C64" t="s">
+        <v>97</v>
+      </c>
+      <c r="D64">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>99</v>
+      </c>
+      <c r="B65" t="s">
+        <v>52</v>
+      </c>
+      <c r="C65" t="s">
+        <v>94</v>
+      </c>
+      <c r="D65">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>100</v>
+      </c>
+      <c r="B66" t="s">
+        <v>101</v>
+      </c>
+      <c r="C66" t="s">
+        <v>102</v>
+      </c>
+      <c r="D66">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>103</v>
+      </c>
+      <c r="B67" t="s">
+        <v>10</v>
+      </c>
+      <c r="C67" t="s">
+        <v>104</v>
+      </c>
+      <c r="D67">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>103</v>
+      </c>
+      <c r="B68" t="s">
+        <v>9</v>
+      </c>
+      <c r="C68" t="s">
+        <v>111</v>
+      </c>
+      <c r="D68">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>103</v>
+      </c>
+      <c r="B69" t="s">
+        <v>96</v>
+      </c>
+      <c r="C69" t="s">
+        <v>105</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>107</v>
+      </c>
+      <c r="B70" t="s">
+        <v>108</v>
+      </c>
+      <c r="C70" t="s">
+        <v>104</v>
+      </c>
+      <c r="D70">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>107</v>
+      </c>
+      <c r="B71" t="s">
+        <v>109</v>
+      </c>
+      <c r="C71" t="s">
+        <v>111</v>
+      </c>
+      <c r="D71">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>107</v>
+      </c>
+      <c r="B72" t="s">
+        <v>51</v>
+      </c>
+      <c r="C72" t="s">
+        <v>105</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>107</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C73" t="s">
+        <v>112</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>114</v>
+      </c>
+      <c r="B74" t="s">
+        <v>115</v>
+      </c>
+      <c r="C74" t="s">
+        <v>117</v>
+      </c>
+      <c r="D74">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>114</v>
+      </c>
+      <c r="B75" t="s">
+        <v>72</v>
+      </c>
+      <c r="C75" t="s">
+        <v>118</v>
+      </c>
+      <c r="D75">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>114</v>
+      </c>
+      <c r="B76" t="s">
+        <v>51</v>
+      </c>
+      <c r="C76" t="s">
+        <v>119</v>
+      </c>
+      <c r="D76">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>114</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C77" t="s">
+        <v>105</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>121</v>
+      </c>
+      <c r="B78" t="s">
+        <v>50</v>
+      </c>
+      <c r="C78" t="s">
+        <v>122</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>124</v>
+      </c>
+      <c r="B79" t="s">
+        <v>108</v>
+      </c>
+      <c r="C79" t="s">
+        <v>138</v>
+      </c>
+      <c r="D79">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>124</v>
+      </c>
+      <c r="B80" t="s">
+        <v>108</v>
+      </c>
+      <c r="C80" t="s">
+        <v>126</v>
+      </c>
+      <c r="D80">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>124</v>
+      </c>
+      <c r="B81" t="s">
+        <v>108</v>
+      </c>
+      <c r="C81" t="s">
+        <v>127</v>
+      </c>
+      <c r="D81">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>124</v>
+      </c>
+      <c r="B82" t="s">
+        <v>125</v>
+      </c>
+      <c r="C82" t="s">
+        <v>128</v>
+      </c>
+      <c r="D82" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>124</v>
+      </c>
+      <c r="B83" t="s">
+        <v>108</v>
+      </c>
+      <c r="C83" t="s">
+        <v>129</v>
+      </c>
+      <c r="D83">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>124</v>
+      </c>
+      <c r="B84" t="s">
+        <v>64</v>
+      </c>
+      <c r="C84" t="s">
+        <v>131</v>
+      </c>
+      <c r="D84">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>124</v>
+      </c>
+      <c r="B85" t="s">
+        <v>64</v>
+      </c>
+      <c r="C85" t="s">
+        <v>132</v>
+      </c>
+      <c r="D85">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>124</v>
+      </c>
+      <c r="B86" t="s">
+        <v>64</v>
+      </c>
+      <c r="C86" t="s">
+        <v>133</v>
+      </c>
+      <c r="D86">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>124</v>
+      </c>
+      <c r="B87" t="s">
+        <v>51</v>
+      </c>
+      <c r="C87" t="s">
+        <v>134</v>
+      </c>
+      <c r="D87">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>135</v>
+      </c>
+      <c r="B88" t="s">
+        <v>51</v>
+      </c>
+      <c r="C88" t="s">
+        <v>136</v>
+      </c>
+      <c r="D88">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>135</v>
+      </c>
+      <c r="B89" t="s">
+        <v>51</v>
+      </c>
+      <c r="C89" t="s">
+        <v>137</v>
+      </c>
+      <c r="D89">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>139</v>
+      </c>
+      <c r="B90" t="s">
+        <v>50</v>
+      </c>
+      <c r="C90" t="s">
+        <v>141</v>
+      </c>
+      <c r="D90">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>139</v>
+      </c>
+      <c r="B91" t="s">
+        <v>108</v>
+      </c>
+      <c r="C91" t="s">
+        <v>142</v>
+      </c>
+      <c r="D91">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>139</v>
+      </c>
+      <c r="B92" t="s">
+        <v>108</v>
+      </c>
+      <c r="C92" t="s">
+        <v>143</v>
+      </c>
+      <c r="D92">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>139</v>
+      </c>
+      <c r="B93" t="s">
+        <v>51</v>
+      </c>
+      <c r="C93" t="s">
+        <v>144</v>
+      </c>
+      <c r="D93">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>139</v>
+      </c>
+      <c r="B94" t="s">
+        <v>64</v>
+      </c>
+      <c r="C94" t="s">
+        <v>145</v>
+      </c>
+      <c r="D94">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>140</v>
+      </c>
+      <c r="B95" t="s">
+        <v>52</v>
+      </c>
+      <c r="C95" t="s">
+        <v>144</v>
+      </c>
+      <c r="D95">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>140</v>
+      </c>
+      <c r="B96" t="s">
+        <v>52</v>
+      </c>
+      <c r="C96" t="s">
+        <v>145</v>
+      </c>
+      <c r="D96">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>146</v>
+      </c>
+      <c r="B97" t="s">
+        <v>108</v>
+      </c>
+      <c r="C97" t="s">
+        <v>141</v>
+      </c>
+      <c r="D97">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>146</v>
+      </c>
+      <c r="B98" t="s">
+        <v>51</v>
+      </c>
+      <c r="C98" t="s">
+        <v>142</v>
+      </c>
+      <c r="D98">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>146</v>
+      </c>
+      <c r="B99" t="s">
+        <v>51</v>
+      </c>
+      <c r="C99" t="s">
+        <v>143</v>
+      </c>
+      <c r="D99">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>146</v>
+      </c>
+      <c r="B100" t="s">
+        <v>51</v>
+      </c>
+      <c r="C100" t="s">
+        <v>147</v>
+      </c>
+      <c r="D100">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>146</v>
+      </c>
+      <c r="B101" t="s">
+        <v>73</v>
+      </c>
+      <c r="C101" t="s">
+        <v>148</v>
+      </c>
+      <c r="D101">
+        <v>450</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: added animations to Zabiegi and PickTreatment.js change: added headers to Cennik items
</commit_message>
<xml_diff>
--- a/backend/data/cennik.xlsx
+++ b/backend/data/cennik.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\StronaMonika\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC225CB-FFAA-4FF1-BC29-0447F4E23759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D81E26C-525A-4377-B4E9-89BF9438E8DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="152">
   <si>
     <t>OPIS</t>
   </si>
@@ -489,6 +489,9 @@
   </si>
   <si>
     <t>Odświeżenie od 1,5 roku do 2 lat od wykonania pierwszego zabiegu</t>
+  </si>
+  <si>
+    <t>Oczy + Twarz</t>
   </si>
 </sst>
 </file>
@@ -2151,7 +2154,7 @@
         <v>108</v>
       </c>
       <c r="C92" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="D92">
         <v>300</v>

</xml_diff>

<commit_message>
feat: added polished style
</commit_message>
<xml_diff>
--- a/backend/data/cennik.xlsx
+++ b/backend/data/cennik.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\StronaMonikaJS\backend\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\StronaMonika\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15DFFC2D-D5BC-4381-AA21-E7B60790A59F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7C2B515-6FE7-4539-888F-B5577567E361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="0" windowWidth="19920" windowHeight="12336" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="146">
   <si>
     <t>OPIS</t>
   </si>
@@ -182,9 +182,6 @@
     <t>65 min</t>
   </si>
   <si>
-    <t>Bez Malowania</t>
-  </si>
-  <si>
     <t>Z malowaniem jeden kolor/odżywka</t>
   </si>
   <si>
@@ -194,51 +191,21 @@
     <t>Manicure Japoński</t>
   </si>
   <si>
-    <t>Regeneracja Płytki Paznokciowej</t>
-  </si>
-  <si>
-    <t>Depilacja Woskiem Karku</t>
-  </si>
-  <si>
-    <t>Depilacja Woskiem Połowy pleców z karkiem/klatką piersiową</t>
-  </si>
-  <si>
     <t>Manicure Hybrydowy</t>
   </si>
   <si>
     <t>90 - 100 min</t>
   </si>
   <si>
-    <t>Baza Hybrydowa</t>
-  </si>
-  <si>
     <t>Z malowaniem na jeden kolor</t>
   </si>
   <si>
-    <t>Z Malowaniem French/Babyboomer</t>
-  </si>
-  <si>
     <t>30 - 40 min</t>
   </si>
   <si>
-    <t>Z Malowaniem Na Jeden Kolor/Odżywka</t>
-  </si>
-  <si>
-    <t>Z Malowaniem French</t>
-  </si>
-  <si>
     <t>100 min</t>
   </si>
   <si>
-    <t>Z Malowaniem Na Jeden Kolor</t>
-  </si>
-  <si>
-    <t>Z Maską w Kremie</t>
-  </si>
-  <si>
-    <t>Z Dodatkowym Peelingiem Chemicznym</t>
-  </si>
-  <si>
     <t>+ 100</t>
   </si>
   <si>
@@ -254,12 +221,6 @@
     <t>+ 20 min</t>
   </si>
   <si>
-    <t>Z Ampułką i Maską Algową</t>
-  </si>
-  <si>
-    <t>Z Dodatkowym Masażem</t>
-  </si>
-  <si>
     <t>+ 20</t>
   </si>
   <si>
@@ -272,12 +233,6 @@
     <t>Twarz</t>
   </si>
   <si>
-    <t>Twarz z Szyją</t>
-  </si>
-  <si>
-    <t>Twarzy, Szyja i Dekolt</t>
-  </si>
-  <si>
     <t>+ 30</t>
   </si>
   <si>
@@ -305,9 +260,6 @@
     <t>Zabieg Nanoigły (Zabieg na Przebarwienia, Blizny, Zmarszczki, Rozszerzone Pory)</t>
   </si>
   <si>
-    <t>Z Jedną Ampułką Nanoigieł</t>
-  </si>
-  <si>
     <t>PqAge (Twarz i Szyja)</t>
   </si>
   <si>
@@ -455,9 +407,6 @@
     <t>Henna rzęs i brwi z regulacją pęsetą/woskiem (komplet)</t>
   </si>
   <si>
-    <t>Dodatkowa Maska Algowa do zabiegu</t>
-  </si>
-  <si>
     <t>Zabieg Oczyszczania Manualnego Twarzy</t>
   </si>
   <si>
@@ -477,6 +426,54 @@
   </si>
   <si>
     <t>Depilacja tułowia</t>
+  </si>
+  <si>
+    <t>Depilacja woskiem karku</t>
+  </si>
+  <si>
+    <t>Depilacja woskiem połowy pleców z karkiem/klatką piersiową</t>
+  </si>
+  <si>
+    <t>Bez malowania</t>
+  </si>
+  <si>
+    <t>Baza hybrydowa</t>
+  </si>
+  <si>
+    <t>Regeneracja płytki paznokciowej</t>
+  </si>
+  <si>
+    <t>Z malowaniem French/Babyboomer</t>
+  </si>
+  <si>
+    <t>Z malowaniem na jeden kolor/odżywka</t>
+  </si>
+  <si>
+    <t>Z malowaniem French</t>
+  </si>
+  <si>
+    <t>Z maską w kremie</t>
+  </si>
+  <si>
+    <t>Z ampułką i maską algową</t>
+  </si>
+  <si>
+    <t>Z dodatkowym peelingiem chemicznym</t>
+  </si>
+  <si>
+    <t>Z dodatkowym masażem</t>
+  </si>
+  <si>
+    <t>Dodatkowa maska algowa do zabiegu</t>
+  </si>
+  <si>
+    <t>Twarz z szyją</t>
+  </si>
+  <si>
+    <t>Twarzy, szyja i dekolt</t>
+  </si>
+  <si>
+    <t>Z jedną ampułką nanoigieł</t>
   </si>
 </sst>
 </file>
@@ -851,15 +848,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED3D7DE2-9127-49D9-96AA-B2504799E15F}">
   <dimension ref="A1:D100"/>
-  <sheetFormatPr defaultColWidth="32" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="32" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="39.109375" customWidth="1"/>
-    <col min="2" max="2" width="17.6640625" customWidth="1"/>
-    <col min="3" max="3" width="49.44140625" customWidth="1"/>
-    <col min="4" max="4" width="18.109375" customWidth="1"/>
+    <col min="1" max="1" width="39.140625" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="49.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -873,7 +870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -881,13 +878,13 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="D2">
         <v>1000</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -895,13 +892,13 @@
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="D3">
         <v>500</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -909,13 +906,13 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D4">
         <v>750</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -923,13 +920,13 @@
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -937,13 +934,13 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="D6">
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -951,13 +948,13 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="D7">
         <v>600</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -965,13 +962,13 @@
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="D8">
         <v>800</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -979,13 +976,13 @@
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -993,13 +990,13 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="D10">
         <v>700</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -1007,13 +1004,13 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="D11">
         <v>900</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -1021,13 +1018,13 @@
         <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="D12">
         <v>500</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -1035,13 +1032,13 @@
         <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="D13">
         <v>500</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -1049,13 +1046,13 @@
         <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="D14">
         <v>700</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -1063,13 +1060,13 @@
         <v>7</v>
       </c>
       <c r="C15" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="D15">
         <v>300</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -1077,13 +1074,13 @@
         <v>7</v>
       </c>
       <c r="C16" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="D16">
         <v>400</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>5</v>
       </c>
@@ -1091,18 +1088,18 @@
         <v>9</v>
       </c>
       <c r="C17" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="C18" t="s">
         <v>10</v>
@@ -1111,12 +1108,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="C19" t="s">
         <v>12</v>
@@ -1125,21 +1122,21 @@
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="C20" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="D20">
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -1153,7 +1150,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -1167,7 +1164,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -1181,7 +1178,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -1195,7 +1192,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>17</v>
       </c>
@@ -1209,7 +1206,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>20</v>
       </c>
@@ -1223,7 +1220,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>20</v>
       </c>
@@ -1237,7 +1234,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -1251,7 +1248,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>22</v>
       </c>
@@ -1265,37 +1262,37 @@
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>146</v>
+        <v>129</v>
       </c>
       <c r="B30" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="C30" t="s">
-        <v>53</v>
+        <v>130</v>
       </c>
       <c r="D30">
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>146</v>
+        <v>129</v>
       </c>
       <c r="B31" t="s">
         <v>34</v>
       </c>
       <c r="C31" t="s">
-        <v>54</v>
+        <v>131</v>
       </c>
       <c r="D31">
         <v>70</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>146</v>
+        <v>129</v>
       </c>
       <c r="B32" t="s">
         <v>39</v>
@@ -1307,37 +1304,37 @@
         <v>100</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>146</v>
+        <v>129</v>
       </c>
       <c r="B33" t="s">
         <v>34</v>
       </c>
       <c r="C33" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="D33">
         <v>100</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="B34" t="s">
         <v>31</v>
       </c>
       <c r="C34" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="D34">
         <v>120</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="B35" t="s">
         <v>32</v>
@@ -1349,9 +1346,9 @@
         <v>170</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="B36" t="s">
         <v>33</v>
@@ -1363,9 +1360,9 @@
         <v>200</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="B37" t="s">
         <v>32</v>
@@ -1377,9 +1374,9 @@
         <v>150</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="B38" t="s">
         <v>34</v>
@@ -1391,9 +1388,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="B39" t="s">
         <v>35</v>
@@ -1405,9 +1402,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="B40" t="s">
         <v>31</v>
@@ -1419,9 +1416,9 @@
         <v>55</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="B41" t="s">
         <v>34</v>
@@ -1433,23 +1430,23 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="B42" t="s">
         <v>33</v>
       </c>
       <c r="C42" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="D42">
         <v>145</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="B43" t="s">
         <v>39</v>
@@ -1461,23 +1458,23 @@
         <v>40</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="B44" t="s">
         <v>41</v>
       </c>
       <c r="C44" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="D44">
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="B45" t="s">
         <v>42</v>
@@ -1489,35 +1486,35 @@
         <v>270</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="B46" t="s">
         <v>39</v>
       </c>
       <c r="C46" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="D46">
         <v>70</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="B47" t="s">
         <v>31</v>
       </c>
       <c r="C47" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
       <c r="D47">
         <v>80</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>45</v>
       </c>
@@ -1525,13 +1522,13 @@
         <v>46</v>
       </c>
       <c r="C48" t="s">
-        <v>48</v>
+        <v>132</v>
       </c>
       <c r="D48">
         <v>90</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>45</v>
       </c>
@@ -1539,13 +1536,13 @@
         <v>32</v>
       </c>
       <c r="C49" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D49">
         <v>100</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>45</v>
       </c>
@@ -1553,707 +1550,707 @@
         <v>47</v>
       </c>
       <c r="C50" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D50">
         <v>120</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B51" t="s">
         <v>32</v>
       </c>
       <c r="C51" t="s">
-        <v>52</v>
+        <v>134</v>
       </c>
       <c r="D51">
         <v>110</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B52" t="s">
         <v>32</v>
       </c>
       <c r="C52" t="s">
-        <v>57</v>
+        <v>133</v>
       </c>
       <c r="D52">
         <v>140</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C53" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D53">
         <v>150</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B54" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C54" t="s">
-        <v>59</v>
+        <v>135</v>
       </c>
       <c r="D54">
         <v>170</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B55" t="s">
         <v>34</v>
       </c>
       <c r="C55" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B56" t="s">
         <v>35</v>
       </c>
       <c r="C56" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="D56">
         <v>20</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B57" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C57" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="D57">
         <v>30</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="B58" t="s">
         <v>31</v>
       </c>
       <c r="C58" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="B59" t="s">
         <v>31</v>
       </c>
       <c r="C59" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="D59">
         <v>70</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="B60" t="s">
         <v>46</v>
       </c>
       <c r="C60" t="s">
-        <v>48</v>
+        <v>132</v>
       </c>
       <c r="D60">
         <v>90</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="B61" t="s">
         <v>32</v>
       </c>
       <c r="C61" t="s">
-        <v>61</v>
+        <v>136</v>
       </c>
       <c r="D61">
         <v>100</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="B62" t="s">
         <v>33</v>
       </c>
       <c r="C62" t="s">
-        <v>62</v>
+        <v>137</v>
       </c>
       <c r="D62">
         <v>120</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="B63" t="s">
         <v>32</v>
       </c>
       <c r="C63" t="s">
-        <v>57</v>
+        <v>133</v>
       </c>
       <c r="D63">
         <v>140</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="B64" t="s">
         <v>41</v>
       </c>
       <c r="C64" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="D64">
         <v>150</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="B65" t="s">
         <v>33</v>
       </c>
       <c r="C65" t="s">
-        <v>62</v>
+        <v>137</v>
       </c>
       <c r="D65">
         <v>170</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="B66" t="s">
         <v>34</v>
       </c>
       <c r="C66" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="B67" t="s">
         <v>7</v>
       </c>
       <c r="C67" t="s">
-        <v>65</v>
+        <v>138</v>
       </c>
       <c r="D67">
         <v>220</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="B68" t="s">
         <v>6</v>
       </c>
       <c r="C68" t="s">
-        <v>72</v>
+        <v>139</v>
       </c>
       <c r="D68">
         <v>260</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>123</v>
+      </c>
+      <c r="B69" t="s">
+        <v>55</v>
+      </c>
+      <c r="C69" t="s">
         <v>140</v>
       </c>
-      <c r="B69" t="s">
-        <v>63</v>
-      </c>
-      <c r="C69" t="s">
-        <v>66</v>
-      </c>
       <c r="D69" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="B70" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C70" t="s">
-        <v>65</v>
+        <v>138</v>
       </c>
       <c r="D70">
         <v>160</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="B71" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C71" t="s">
-        <v>72</v>
+        <v>139</v>
       </c>
       <c r="D71">
         <v>200</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="B72" t="s">
         <v>32</v>
       </c>
       <c r="C72" t="s">
-        <v>66</v>
+        <v>140</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="C73" t="s">
-        <v>73</v>
+        <v>141</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="B74" t="s">
         <v>31</v>
       </c>
       <c r="C74" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="B75" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="C75" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="D75">
         <v>190</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="B76" t="s">
         <v>46</v>
       </c>
       <c r="C76" t="s">
-        <v>78</v>
+        <v>143</v>
       </c>
       <c r="D76">
         <v>200</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="B77" t="s">
         <v>32</v>
       </c>
       <c r="C77" t="s">
-        <v>79</v>
+        <v>144</v>
       </c>
       <c r="D77">
         <v>250</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="C78" t="s">
-        <v>66</v>
+        <v>140</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B79" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C79" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="D79">
         <v>300</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B80" t="s">
+        <v>58</v>
+      </c>
+      <c r="C80" t="s">
         <v>69</v>
-      </c>
-      <c r="C80" t="s">
-        <v>84</v>
       </c>
       <c r="D80">
         <v>300</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B81" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C81" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="D81">
         <v>300</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B82" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="C82" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="D82" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B83" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C83" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="D83">
         <v>250</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B84" t="s">
         <v>41</v>
       </c>
       <c r="C84" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="D84">
         <v>350</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B85" t="s">
         <v>41</v>
       </c>
       <c r="C85" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="D85">
         <v>300</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B86" t="s">
         <v>41</v>
       </c>
       <c r="C86" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="D86">
         <v>250</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B87" t="s">
         <v>32</v>
       </c>
       <c r="C87" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="D87">
         <v>220</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="B88" t="s">
         <v>32</v>
       </c>
       <c r="C88" t="s">
-        <v>89</v>
+        <v>145</v>
       </c>
       <c r="D88">
         <v>400</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="B89" t="s">
         <v>31</v>
       </c>
       <c r="C89" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="D89">
         <v>220</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="B90" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C90" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="D90">
         <v>250</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="B91" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C91" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="D91">
         <v>300</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="B92" t="s">
         <v>32</v>
       </c>
       <c r="C92" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="D92">
         <v>330</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="B93" t="s">
         <v>41</v>
       </c>
       <c r="C93" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="D93">
         <v>350</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>143</v>
+        <v>126</v>
       </c>
       <c r="B94" t="s">
         <v>33</v>
       </c>
       <c r="C94" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="D94">
         <v>450</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>143</v>
+        <v>126</v>
       </c>
       <c r="B95" t="s">
         <v>33</v>
       </c>
       <c r="C95" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="D95">
         <v>550</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>144</v>
+        <v>127</v>
       </c>
       <c r="B96" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C96" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="D96">
         <v>280</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>144</v>
+        <v>127</v>
       </c>
       <c r="B97" t="s">
         <v>32</v>
       </c>
       <c r="C97" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="D97">
         <v>300</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>144</v>
+        <v>127</v>
       </c>
       <c r="B98" t="s">
         <v>32</v>
       </c>
       <c r="C98" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="D98">
         <v>350</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>144</v>
+        <v>127</v>
       </c>
       <c r="B99" t="s">
         <v>32</v>
       </c>
       <c r="C99" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="D99">
         <v>400</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>144</v>
+        <v>127</v>
       </c>
       <c r="B100" t="s">
         <v>47</v>
       </c>
       <c r="C100" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="D100">
         <v>450</v>

</xml_diff>

<commit_message>
feat: added minor changes
</commit_message>
<xml_diff>
--- a/backend/data/cennik.xlsx
+++ b/backend/data/cennik.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\StronaMonika\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7C2B515-6FE7-4539-888F-B5577567E361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F125FD6-81E6-4561-8AF0-E5AA4BAB55B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="146">
   <si>
     <t>OPIS</t>
   </si>
@@ -473,7 +473,7 @@
     <t>Twarzy, szyja i dekolt</t>
   </si>
   <si>
-    <t>Z jedną ampułką nanoigieł</t>
+    <t>Twarz z Szyją/Dekolt</t>
   </si>
 </sst>
 </file>
@@ -847,7 +847,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED3D7DE2-9127-49D9-96AA-B2504799E15F}">
-  <dimension ref="A1:D100"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr defaultColWidth="32" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39.140625" customWidth="1"/>
@@ -2085,21 +2085,21 @@
         <v>145</v>
       </c>
       <c r="D88">
-        <v>400</v>
+        <v>350</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>125</v>
+        <v>73</v>
       </c>
       <c r="B89" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C89" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D89">
-        <v>220</v>
+        <v>450</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -2107,13 +2107,13 @@
         <v>125</v>
       </c>
       <c r="B90" t="s">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="C90" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D90">
-        <v>250</v>
+        <v>220</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -2124,10 +2124,10 @@
         <v>58</v>
       </c>
       <c r="C91" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="D91">
-        <v>300</v>
+        <v>250</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -2135,13 +2135,13 @@
         <v>125</v>
       </c>
       <c r="B92" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="C92" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D92">
-        <v>330</v>
+        <v>300</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -2149,27 +2149,27 @@
         <v>125</v>
       </c>
       <c r="B93" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="C93" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D93">
-        <v>350</v>
+        <v>330</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B94" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="C94" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D94">
-        <v>450</v>
+        <v>350</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -2180,24 +2180,24 @@
         <v>33</v>
       </c>
       <c r="C95" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D95">
-        <v>550</v>
+        <v>450</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B96" t="s">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="C96" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D96">
-        <v>280</v>
+        <v>550</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -2205,13 +2205,13 @@
         <v>127</v>
       </c>
       <c r="B97" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="C97" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D97">
-        <v>300</v>
+        <v>280</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -2222,10 +2222,10 @@
         <v>32</v>
       </c>
       <c r="C98" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D98">
-        <v>350</v>
+        <v>300</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -2236,10 +2236,10 @@
         <v>32</v>
       </c>
       <c r="C99" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D99">
-        <v>400</v>
+        <v>350</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -2247,12 +2247,26 @@
         <v>127</v>
       </c>
       <c r="B100" t="s">
+        <v>32</v>
+      </c>
+      <c r="C100" t="s">
+        <v>80</v>
+      </c>
+      <c r="D100">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>127</v>
+      </c>
+      <c r="B101" t="s">
         <v>47</v>
       </c>
-      <c r="C100" t="s">
+      <c r="C101" t="s">
         <v>81</v>
       </c>
-      <c r="D100">
+      <c r="D101">
         <v>450</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: added waiting for content load on all sites
</commit_message>
<xml_diff>
--- a/backend/data/cennik.xlsx
+++ b/backend/data/cennik.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\StronaMonika\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F125FD6-81E6-4561-8AF0-E5AA4BAB55B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E076B86-81A7-43DC-BB9D-5C9DD83330BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
+    <workbookView xWindow="-14505" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="144">
   <si>
     <t>OPIS</t>
   </si>
@@ -92,12 +92,6 @@
     <t>Depilacja pach</t>
   </si>
   <si>
-    <t>Depilacja woskiem pachy damskie</t>
-  </si>
-  <si>
-    <t>Depilacja woskiem pachy męskie</t>
-  </si>
-  <si>
     <t>Depilacja rąk</t>
   </si>
   <si>
@@ -182,12 +176,6 @@
     <t>65 min</t>
   </si>
   <si>
-    <t>Z malowaniem jeden kolor/odżywka</t>
-  </si>
-  <si>
-    <t>Z malowaniem french</t>
-  </si>
-  <si>
     <t>Manicure Japoński</t>
   </si>
   <si>
@@ -251,9 +239,6 @@
     <t>RETIX C EYE (Oczy)</t>
   </si>
   <si>
-    <t>Kwasy RETIX C (Twarz, Szyja lub Dekolt)</t>
-  </si>
-  <si>
     <t>180 - 300</t>
   </si>
   <si>
@@ -359,9 +344,6 @@
     <t>Dodatkowa korekta brwi. Druga korekta nie wliczona w cenę podstawową</t>
   </si>
   <si>
-    <t>Dodatkowa korekta kreska. Druga korekta nie wliczona w cenę podstawową</t>
-  </si>
-  <si>
     <t>Do 2 lat od wykonania pierwszego zabiegu - odświeżenie</t>
   </si>
   <si>
@@ -474,6 +456,18 @@
   </si>
   <si>
     <t>Twarz z Szyją/Dekolt</t>
+  </si>
+  <si>
+    <t>Monokwasy (Twarz, Szyja lub Dekolt)</t>
+  </si>
+  <si>
+    <t>Depilacja woskiem pach damskich</t>
+  </si>
+  <si>
+    <t>Depilacja woskiem pach męskich</t>
+  </si>
+  <si>
+    <t>Dodatkowa korekta kreski. Druga korekta nie wliczona w cenę podstawową</t>
   </si>
 </sst>
 </file>
@@ -861,7 +855,7 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -878,7 +872,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="D2">
         <v>1000</v>
@@ -892,7 +886,7 @@
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D3">
         <v>500</v>
@@ -906,7 +900,7 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D4">
         <v>750</v>
@@ -920,10 +914,10 @@
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -934,7 +928,7 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D6">
         <v>1000</v>
@@ -948,7 +942,7 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="D7">
         <v>600</v>
@@ -962,7 +956,7 @@
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D8">
         <v>800</v>
@@ -976,10 +970,10 @@
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -990,7 +984,7 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D10">
         <v>700</v>
@@ -1004,7 +998,7 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="D11">
         <v>900</v>
@@ -1018,7 +1012,7 @@
         <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D12">
         <v>500</v>
@@ -1032,7 +1026,7 @@
         <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="D13">
         <v>500</v>
@@ -1046,7 +1040,7 @@
         <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D14">
         <v>700</v>
@@ -1060,7 +1054,7 @@
         <v>7</v>
       </c>
       <c r="C15" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="D15">
         <v>300</v>
@@ -1074,7 +1068,7 @@
         <v>7</v>
       </c>
       <c r="C16" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="D16">
         <v>400</v>
@@ -1088,10 +1082,10 @@
         <v>9</v>
       </c>
       <c r="C17" t="s">
-        <v>107</v>
+        <v>143</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1099,7 +1093,7 @@
         <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C18" t="s">
         <v>10</v>
@@ -1113,7 +1107,7 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C19" t="s">
         <v>12</v>
@@ -1127,10 +1121,10 @@
         <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C20" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D20">
         <v>50</v>
@@ -1141,7 +1135,7 @@
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C21" t="s">
         <v>14</v>
@@ -1155,7 +1149,7 @@
         <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C22" t="s">
         <v>15</v>
@@ -1169,7 +1163,7 @@
         <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C23" t="s">
         <v>16</v>
@@ -1183,10 +1177,10 @@
         <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C24" t="s">
-        <v>18</v>
+        <v>141</v>
       </c>
       <c r="D24">
         <v>50</v>
@@ -1197,10 +1191,10 @@
         <v>17</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>19</v>
+        <v>142</v>
       </c>
       <c r="D25">
         <v>60</v>
@@ -1208,13 +1202,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C26" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D26">
         <v>60</v>
@@ -1222,13 +1216,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B27" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C27" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D27">
         <v>80</v>
@@ -1236,13 +1230,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D28">
         <v>75</v>
@@ -1250,13 +1244,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B29" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C29" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D29">
         <v>120</v>
@@ -1264,13 +1258,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B30" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C30" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="D30">
         <v>40</v>
@@ -1278,13 +1272,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B31" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C31" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="D31">
         <v>70</v>
@@ -1292,13 +1286,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B32" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C32" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D32">
         <v>100</v>
@@ -1306,13 +1300,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B33" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C33" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="D33">
         <v>100</v>
@@ -1320,13 +1314,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B34" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C34" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D34">
         <v>120</v>
@@ -1334,13 +1328,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B35" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C35" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D35">
         <v>170</v>
@@ -1348,13 +1342,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B36" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C36" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D36">
         <v>200</v>
@@ -1362,13 +1356,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B37" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C37" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D37">
         <v>150</v>
@@ -1376,13 +1370,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B38" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C38" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D38">
         <v>60</v>
@@ -1390,13 +1384,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B39" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C39" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D39">
         <v>35</v>
@@ -1404,13 +1398,13 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B40" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C40" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D40">
         <v>55</v>
@@ -1418,13 +1412,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B41" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C41" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D41">
         <v>40</v>
@@ -1432,13 +1426,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B42" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C42" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D42">
         <v>145</v>
@@ -1446,13 +1440,13 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B43" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C43" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D43">
         <v>40</v>
@@ -1460,13 +1454,13 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B44" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C44" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="D44">
         <v>145</v>
@@ -1474,13 +1468,13 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C45" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D45">
         <v>270</v>
@@ -1488,13 +1482,13 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B46" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C46" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D46">
         <v>70</v>
@@ -1502,13 +1496,13 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B47" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C47" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="D47">
         <v>80</v>
@@ -1516,13 +1510,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B48" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C48" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D48">
         <v>90</v>
@@ -1530,13 +1524,13 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B49" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C49" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D49">
         <v>100</v>
@@ -1544,13 +1538,13 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>43</v>
+      </c>
+      <c r="B50" t="s">
         <v>45</v>
       </c>
-      <c r="B50" t="s">
-        <v>47</v>
-      </c>
       <c r="C50" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="D50">
         <v>120</v>
@@ -1558,13 +1552,13 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B51" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C51" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="D51">
         <v>110</v>
@@ -1572,13 +1566,13 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B52" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C52" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D52">
         <v>140</v>
@@ -1586,13 +1580,13 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B53" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C53" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D53">
         <v>150</v>
@@ -1600,13 +1594,13 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B54" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C54" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D54">
         <v>170</v>
@@ -1614,27 +1608,27 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B55" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C55" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B56" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C56" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D56">
         <v>20</v>
@@ -1642,13 +1636,13 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B57" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C57" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D57">
         <v>30</v>
@@ -1656,27 +1650,27 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="B58" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C58" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="B59" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C59" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="D59">
         <v>70</v>
@@ -1684,13 +1678,13 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="B60" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C60" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D60">
         <v>90</v>
@@ -1698,13 +1692,13 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="B61" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C61" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="D61">
         <v>100</v>
@@ -1712,13 +1706,13 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="B62" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C62" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="D62">
         <v>120</v>
@@ -1726,13 +1720,13 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B63" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C63" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D63">
         <v>140</v>
@@ -1740,13 +1734,13 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B64" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C64" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D64">
         <v>150</v>
@@ -1754,13 +1748,13 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B65" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C65" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="D65">
         <v>170</v>
@@ -1768,27 +1762,27 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B66" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C66" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B67" t="s">
         <v>7</v>
       </c>
       <c r="C67" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="D67">
         <v>220</v>
@@ -1796,13 +1790,13 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B68" t="s">
         <v>6</v>
       </c>
       <c r="C68" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D68">
         <v>260</v>
@@ -1810,27 +1804,27 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B69" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C69" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B70" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C70" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="D70">
         <v>160</v>
@@ -1838,13 +1832,13 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B71" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C71" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D71">
         <v>200</v>
@@ -1852,55 +1846,55 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B72" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C72" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>53</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C73" t="s">
+        <v>135</v>
+      </c>
+      <c r="D73" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C73" t="s">
-        <v>141</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B74" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C74" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B75" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C75" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D75">
         <v>190</v>
@@ -1908,13 +1902,13 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B76" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C76" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="D76">
         <v>200</v>
@@ -1922,13 +1916,13 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B77" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C77" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="D77">
         <v>250</v>
@@ -1936,27 +1930,27 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C78" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B79" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C79" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D79">
         <v>300</v>
@@ -1964,13 +1958,13 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B80" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C80" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D80">
         <v>300</v>
@@ -1978,13 +1972,13 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B81" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C81" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D81">
         <v>300</v>
@@ -1992,27 +1986,27 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>63</v>
+      </c>
+      <c r="B82" t="s">
+        <v>64</v>
+      </c>
+      <c r="C82" t="s">
+        <v>140</v>
+      </c>
+      <c r="D82" t="s">
         <v>67</v>
-      </c>
-      <c r="B82" t="s">
-        <v>68</v>
-      </c>
-      <c r="C82" t="s">
-        <v>71</v>
-      </c>
-      <c r="D82" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B83" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C83" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D83">
         <v>250</v>
@@ -2020,13 +2014,13 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B84" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C84" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="D84">
         <v>350</v>
@@ -2034,13 +2028,13 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B85" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C85" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D85">
         <v>300</v>
@@ -2048,13 +2042,13 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B86" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C86" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D86">
         <v>250</v>
@@ -2062,13 +2056,13 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B87" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C87" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="D87">
         <v>220</v>
@@ -2076,13 +2070,13 @@
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B88" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C88" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="D88">
         <v>350</v>
@@ -2090,13 +2084,13 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B89" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C89" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D89">
         <v>450</v>
@@ -2104,13 +2098,13 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B90" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C90" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="D90">
         <v>220</v>
@@ -2118,13 +2112,13 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B91" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C91" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="D91">
         <v>250</v>
@@ -2132,13 +2126,13 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B92" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C92" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D92">
         <v>300</v>
@@ -2146,13 +2140,13 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B93" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C93" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D93">
         <v>330</v>
@@ -2160,13 +2154,13 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B94" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C94" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D94">
         <v>350</v>
@@ -2174,13 +2168,13 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="B95" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C95" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D95">
         <v>450</v>
@@ -2188,13 +2182,13 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="B96" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C96" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D96">
         <v>550</v>
@@ -2202,13 +2196,13 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B97" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C97" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="D97">
         <v>280</v>
@@ -2216,13 +2210,13 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B98" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C98" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="D98">
         <v>300</v>
@@ -2230,13 +2224,13 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B99" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C99" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D99">
         <v>350</v>
@@ -2244,13 +2238,13 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B100" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C100" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D100">
         <v>400</v>
@@ -2258,13 +2252,13 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B101" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C101" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D101">
         <v>450</v>

</xml_diff>

<commit_message>
feat: changing last styles
</commit_message>
<xml_diff>
--- a/backend/data/cennik.xlsx
+++ b/backend/data/cennik.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\StronaMonika\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{441FBFAD-ED14-4A5B-BD72-04DDC34BA39C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{455FFD8A-A8C2-4BB6-8C7C-23AFB0ABF20D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14505" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="142">
   <si>
     <t>OPIS</t>
   </si>
@@ -410,9 +410,6 @@
     <t>Depilacja woskiem karku</t>
   </si>
   <si>
-    <t>Depilacja woskiem połowy pleców z karkiem/klatką piersiową</t>
-  </si>
-  <si>
     <t>Bez malowania</t>
   </si>
   <si>
@@ -459,13 +456,19 @@
   </si>
   <si>
     <t>Dodatkowy peeling chemiczny</t>
+  </si>
+  <si>
+    <t>Depilacja woskiem połowy pleców z karkiem</t>
+  </si>
+  <si>
+    <t>Depilacja klatki piersiowej</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -832,16 +835,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED3D7DE2-9127-49D9-96AA-B2504799E15F}">
-  <dimension ref="A1:D101"/>
-  <sheetFormatPr defaultColWidth="32" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D102"/>
+  <sheetFormatPr defaultColWidth="32" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="39.140625" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
-    <col min="3" max="3" width="49.42578125" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="1" max="1" width="39.125" customWidth="1"/>
+    <col min="2" max="2" width="17.75" customWidth="1"/>
+    <col min="3" max="3" width="49.375" customWidth="1"/>
+    <col min="4" max="4" width="18.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -855,7 +858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -869,7 +872,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -883,7 +886,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -897,7 +900,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -911,7 +914,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -925,7 +928,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -939,7 +942,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -953,7 +956,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -967,7 +970,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -981,7 +984,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -995,7 +998,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -1009,7 +1012,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -1023,7 +1026,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -1037,7 +1040,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -1051,7 +1054,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -1065,7 +1068,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4">
       <c r="A17" t="s">
         <v>5</v>
       </c>
@@ -1073,13 +1076,13 @@
         <v>9</v>
       </c>
       <c r="C17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -1093,7 +1096,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -1107,7 +1110,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4">
       <c r="A20" t="s">
         <v>11</v>
       </c>
@@ -1121,7 +1124,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -1135,7 +1138,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -1149,7 +1152,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -1163,7 +1166,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -1171,13 +1174,13 @@
         <v>33</v>
       </c>
       <c r="C24" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D24">
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4">
       <c r="A25" t="s">
         <v>17</v>
       </c>
@@ -1185,13 +1188,13 @@
         <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D25">
         <v>60</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4">
       <c r="A26" t="s">
         <v>18</v>
       </c>
@@ -1205,7 +1208,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4">
       <c r="A27" t="s">
         <v>18</v>
       </c>
@@ -1219,7 +1222,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4">
       <c r="A28" t="s">
         <v>20</v>
       </c>
@@ -1233,7 +1236,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4">
       <c r="A29" t="s">
         <v>20</v>
       </c>
@@ -1247,7 +1250,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4">
       <c r="A30" t="s">
         <v>122</v>
       </c>
@@ -1261,7 +1264,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4">
       <c r="A31" t="s">
         <v>122</v>
       </c>
@@ -1269,295 +1272,295 @@
         <v>32</v>
       </c>
       <c r="C31" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="D31">
         <v>70</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4">
       <c r="A32" t="s">
         <v>122</v>
       </c>
       <c r="B32" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C32" t="s">
-        <v>24</v>
+        <v>141</v>
       </c>
       <c r="D32">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
       <c r="A33" t="s">
         <v>122</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C33" t="s">
-        <v>80</v>
+        <v>24</v>
       </c>
       <c r="D33">
         <v>100</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>82</v>
+        <v>122</v>
       </c>
       <c r="B34" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C34" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D34">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
       <c r="A35" t="s">
         <v>82</v>
       </c>
       <c r="B35" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C35" t="s">
-        <v>25</v>
+        <v>83</v>
       </c>
       <c r="D35">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
       <c r="A36" t="s">
         <v>82</v>
       </c>
       <c r="B36" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C36" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D36">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
       <c r="A37" t="s">
         <v>82</v>
       </c>
       <c r="B37" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C37" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D37">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
       <c r="A38" t="s">
         <v>82</v>
       </c>
       <c r="B38" t="s">
+        <v>30</v>
+      </c>
+      <c r="C38" t="s">
+        <v>27</v>
+      </c>
+      <c r="D38">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" t="s">
+        <v>82</v>
+      </c>
+      <c r="B39" t="s">
         <v>32</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C39" t="s">
         <v>28</v>
       </c>
-      <c r="D38">
+      <c r="D39">
         <v>60</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>121</v>
-      </c>
-      <c r="B39" t="s">
-        <v>33</v>
-      </c>
-      <c r="C39" t="s">
-        <v>34</v>
-      </c>
-      <c r="D39">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4">
       <c r="A40" t="s">
         <v>121</v>
       </c>
       <c r="B40" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C40" t="s">
+        <v>34</v>
+      </c>
+      <c r="D40">
         <v>35</v>
       </c>
-      <c r="D40">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:4">
       <c r="A41" t="s">
         <v>121</v>
       </c>
       <c r="B41" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C41" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D41">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
       <c r="A42" t="s">
         <v>121</v>
       </c>
       <c r="B42" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C42" t="s">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="D42">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
       <c r="A43" t="s">
         <v>121</v>
       </c>
       <c r="B43" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C43" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="D43">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
       <c r="A44" t="s">
         <v>121</v>
       </c>
       <c r="B44" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C44" t="s">
-        <v>85</v>
+        <v>38</v>
       </c>
       <c r="D44">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
       <c r="A45" t="s">
         <v>121</v>
       </c>
       <c r="B45" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C45" t="s">
-        <v>41</v>
+        <v>85</v>
       </c>
       <c r="D45">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
       <c r="A46" t="s">
         <v>121</v>
       </c>
       <c r="B46" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C46" t="s">
-        <v>114</v>
+        <v>41</v>
       </c>
       <c r="D46">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
       <c r="A47" t="s">
         <v>121</v>
       </c>
       <c r="B47" t="s">
+        <v>37</v>
+      </c>
+      <c r="C47" t="s">
+        <v>114</v>
+      </c>
+      <c r="D47">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" t="s">
+        <v>121</v>
+      </c>
+      <c r="B48" t="s">
         <v>29</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C48" t="s">
         <v>115</v>
       </c>
-      <c r="D47">
+      <c r="D48">
         <v>80</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>43</v>
-      </c>
-      <c r="B48" t="s">
-        <v>44</v>
-      </c>
-      <c r="C48" t="s">
-        <v>125</v>
-      </c>
-      <c r="D48">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4">
       <c r="A49" t="s">
         <v>43</v>
       </c>
       <c r="B49" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C49" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="D49">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
       <c r="A50" t="s">
         <v>43</v>
       </c>
       <c r="B50" t="s">
+        <v>30</v>
+      </c>
+      <c r="C50" t="s">
+        <v>128</v>
+      </c>
+      <c r="D50">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" t="s">
+        <v>43</v>
+      </c>
+      <c r="B51" t="s">
         <v>45</v>
       </c>
-      <c r="C50" t="s">
-        <v>130</v>
-      </c>
-      <c r="D50">
+      <c r="C51" t="s">
+        <v>129</v>
+      </c>
+      <c r="D51">
         <v>120</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+    <row r="52" spans="1:4">
+      <c r="A52" t="s">
         <v>46</v>
-      </c>
-      <c r="B51" t="s">
-        <v>30</v>
-      </c>
-      <c r="C51" t="s">
-        <v>127</v>
-      </c>
-      <c r="D51">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>47</v>
       </c>
       <c r="B52" t="s">
         <v>30</v>
@@ -1566,24 +1569,24 @@
         <v>126</v>
       </c>
       <c r="D52">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
       <c r="A53" t="s">
         <v>47</v>
       </c>
       <c r="B53" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="C53" t="s">
-        <v>49</v>
+        <v>125</v>
       </c>
       <c r="D53">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
       <c r="A54" t="s">
         <v>47</v>
       </c>
@@ -1591,69 +1594,69 @@
         <v>48</v>
       </c>
       <c r="C54" t="s">
-        <v>128</v>
+        <v>49</v>
       </c>
       <c r="D54">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
       <c r="A55" t="s">
         <v>47</v>
       </c>
       <c r="B55" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="C55" t="s">
-        <v>110</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+      <c r="D55">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
       <c r="A56" t="s">
         <v>47</v>
       </c>
       <c r="B56" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C56" t="s">
-        <v>112</v>
-      </c>
-      <c r="D56">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
       <c r="A57" t="s">
         <v>47</v>
       </c>
       <c r="B57" t="s">
+        <v>33</v>
+      </c>
+      <c r="C57" t="s">
+        <v>112</v>
+      </c>
+      <c r="D57">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" t="s">
+        <v>47</v>
+      </c>
+      <c r="B58" t="s">
         <v>50</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C58" t="s">
         <v>113</v>
       </c>
-      <c r="D57">
+      <c r="D58">
         <v>30</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>108</v>
-      </c>
-      <c r="B58" t="s">
-        <v>29</v>
-      </c>
-      <c r="C58" t="s">
-        <v>106</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4">
       <c r="A59" t="s">
         <v>108</v>
       </c>
@@ -1661,293 +1664,293 @@
         <v>29</v>
       </c>
       <c r="C59" t="s">
-        <v>107</v>
-      </c>
-      <c r="D59">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
       <c r="A60" t="s">
         <v>108</v>
       </c>
       <c r="B60" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="C60" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="D60">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
       <c r="A61" t="s">
         <v>108</v>
       </c>
       <c r="B61" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C61" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="D61">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
       <c r="A62" t="s">
         <v>108</v>
       </c>
       <c r="B62" t="s">
+        <v>30</v>
+      </c>
+      <c r="C62" t="s">
+        <v>128</v>
+      </c>
+      <c r="D62">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" t="s">
+        <v>108</v>
+      </c>
+      <c r="B63" t="s">
         <v>31</v>
       </c>
-      <c r="C62" t="s">
-        <v>130</v>
-      </c>
-      <c r="D62">
+      <c r="C63" t="s">
+        <v>129</v>
+      </c>
+      <c r="D63">
         <v>120</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>105</v>
-      </c>
-      <c r="B63" t="s">
-        <v>30</v>
-      </c>
-      <c r="C63" t="s">
-        <v>126</v>
-      </c>
-      <c r="D63">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4">
       <c r="A64" t="s">
         <v>105</v>
       </c>
       <c r="B64" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C64" t="s">
-        <v>49</v>
+        <v>125</v>
       </c>
       <c r="D64">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
       <c r="A65" t="s">
         <v>105</v>
       </c>
       <c r="B65" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="C65" t="s">
-        <v>130</v>
+        <v>49</v>
       </c>
       <c r="D65">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
       <c r="A66" t="s">
         <v>105</v>
       </c>
       <c r="B66" t="s">
+        <v>31</v>
+      </c>
+      <c r="C66" t="s">
+        <v>129</v>
+      </c>
+      <c r="D66">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" t="s">
+        <v>105</v>
+      </c>
+      <c r="B67" t="s">
         <v>32</v>
       </c>
-      <c r="C66" t="s">
+      <c r="C67" t="s">
         <v>106</v>
       </c>
-      <c r="D66" s="1" t="s">
+      <c r="D67" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>116</v>
-      </c>
-      <c r="B67" t="s">
-        <v>7</v>
-      </c>
-      <c r="C67" t="s">
-        <v>131</v>
-      </c>
-      <c r="D67">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4">
       <c r="A68" t="s">
         <v>116</v>
       </c>
       <c r="B68" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C68" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D68">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
       <c r="A69" t="s">
         <v>116</v>
       </c>
       <c r="B69" t="s">
+        <v>6</v>
+      </c>
+      <c r="C69" t="s">
+        <v>131</v>
+      </c>
+      <c r="D69">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" t="s">
+        <v>116</v>
+      </c>
+      <c r="B70" t="s">
         <v>51</v>
       </c>
-      <c r="C69" t="s">
-        <v>140</v>
-      </c>
-      <c r="D69" s="1" t="s">
+      <c r="C70" t="s">
+        <v>139</v>
+      </c>
+      <c r="D70" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>53</v>
-      </c>
-      <c r="B70" t="s">
-        <v>54</v>
-      </c>
-      <c r="C70" t="s">
-        <v>131</v>
-      </c>
-      <c r="D70">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4">
       <c r="A71" t="s">
         <v>53</v>
       </c>
       <c r="B71" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C71" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D71">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
       <c r="A72" t="s">
         <v>53</v>
       </c>
       <c r="B72" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="C72" t="s">
-        <v>140</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+      <c r="D72">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
       <c r="A73" t="s">
         <v>53</v>
       </c>
-      <c r="B73" s="1" t="s">
-        <v>56</v>
+      <c r="B73" t="s">
+        <v>30</v>
       </c>
       <c r="C73" t="s">
         <v>139</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
       <c r="A74" t="s">
         <v>53</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B74" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C74" t="s">
+        <v>138</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4">
+      <c r="A75" t="s">
+        <v>53</v>
+      </c>
+      <c r="B75" t="s">
         <v>29</v>
       </c>
-      <c r="C74" t="s">
-        <v>133</v>
-      </c>
-      <c r="D74" s="1" t="s">
+      <c r="C75" t="s">
+        <v>132</v>
+      </c>
+      <c r="D75" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>117</v>
-      </c>
-      <c r="B75" t="s">
-        <v>58</v>
-      </c>
-      <c r="C75" t="s">
-        <v>60</v>
-      </c>
-      <c r="D75">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4">
       <c r="A76" t="s">
         <v>117</v>
       </c>
       <c r="B76" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="C76" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="D76">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
       <c r="A77" t="s">
         <v>117</v>
       </c>
       <c r="B77" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C77" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D77">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
       <c r="A78" t="s">
         <v>117</v>
       </c>
-      <c r="B78" s="1" t="s">
+      <c r="B78" t="s">
+        <v>30</v>
+      </c>
+      <c r="C78" t="s">
+        <v>76</v>
+      </c>
+      <c r="D78">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4">
+      <c r="A79" t="s">
+        <v>117</v>
+      </c>
+      <c r="B79" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C78" t="s">
-        <v>140</v>
-      </c>
-      <c r="D78" s="1" t="s">
+      <c r="C79" t="s">
+        <v>139</v>
+      </c>
+      <c r="D79" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>63</v>
-      </c>
-      <c r="B79" t="s">
-        <v>54</v>
-      </c>
-      <c r="C79" t="s">
-        <v>69</v>
-      </c>
-      <c r="D79">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4">
       <c r="A80" t="s">
         <v>63</v>
       </c>
@@ -1955,13 +1958,13 @@
         <v>54</v>
       </c>
       <c r="C80" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D80">
         <v>300</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4">
       <c r="A81" t="s">
         <v>63</v>
       </c>
@@ -1969,55 +1972,55 @@
         <v>54</v>
       </c>
       <c r="C81" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D81">
         <v>300</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4">
       <c r="A82" t="s">
         <v>63</v>
       </c>
       <c r="B82" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C82" t="s">
-        <v>135</v>
-      </c>
-      <c r="D82" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+      <c r="D82">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4">
       <c r="A83" t="s">
         <v>63</v>
       </c>
       <c r="B83" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="C83" t="s">
-        <v>90</v>
-      </c>
-      <c r="D83">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+      <c r="D83" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4">
       <c r="A84" t="s">
         <v>63</v>
       </c>
       <c r="B84" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="C84" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D84">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4">
       <c r="A85" t="s">
         <v>63</v>
       </c>
@@ -2025,13 +2028,13 @@
         <v>39</v>
       </c>
       <c r="C85" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D85">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4">
       <c r="A86" t="s">
         <v>63</v>
       </c>
@@ -2039,41 +2042,41 @@
         <v>39</v>
       </c>
       <c r="C86" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D86">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4">
       <c r="A87" t="s">
         <v>63</v>
       </c>
       <c r="B87" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C87" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D87">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
       <c r="A88" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B88" t="s">
         <v>30</v>
       </c>
       <c r="C88" t="s">
-        <v>134</v>
+        <v>86</v>
       </c>
       <c r="D88">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4">
       <c r="A89" t="s">
         <v>68</v>
       </c>
@@ -2081,41 +2084,41 @@
         <v>30</v>
       </c>
       <c r="C89" t="s">
+        <v>133</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4">
+      <c r="A90" t="s">
+        <v>68</v>
+      </c>
+      <c r="B90" t="s">
+        <v>30</v>
+      </c>
+      <c r="C90" t="s">
         <v>76</v>
       </c>
-      <c r="D89">
+      <c r="D90">
         <v>450</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>118</v>
-      </c>
-      <c r="B90" t="s">
-        <v>29</v>
-      </c>
-      <c r="C90" t="s">
-        <v>70</v>
-      </c>
-      <c r="D90">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4">
       <c r="A91" t="s">
         <v>118</v>
       </c>
       <c r="B91" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="C91" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D91">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4">
       <c r="A92" t="s">
         <v>118</v>
       </c>
@@ -2123,55 +2126,55 @@
         <v>54</v>
       </c>
       <c r="C92" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D92">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
       <c r="A93" t="s">
         <v>118</v>
       </c>
       <c r="B93" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C93" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D93">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4">
       <c r="A94" t="s">
         <v>118</v>
       </c>
       <c r="B94" t="s">
+        <v>30</v>
+      </c>
+      <c r="C94" t="s">
+        <v>73</v>
+      </c>
+      <c r="D94">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4">
+      <c r="A95" t="s">
+        <v>118</v>
+      </c>
+      <c r="B95" t="s">
         <v>39</v>
       </c>
-      <c r="C94" t="s">
+      <c r="C95" t="s">
         <v>74</v>
       </c>
-      <c r="D94">
+      <c r="D95">
         <v>350</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>119</v>
-      </c>
-      <c r="B95" t="s">
-        <v>31</v>
-      </c>
-      <c r="C95" t="s">
-        <v>73</v>
-      </c>
-      <c r="D95">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4">
       <c r="A96" t="s">
         <v>119</v>
       </c>
@@ -2179,41 +2182,41 @@
         <v>31</v>
       </c>
       <c r="C96" t="s">
+        <v>73</v>
+      </c>
+      <c r="D96">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4">
+      <c r="A97" t="s">
+        <v>119</v>
+      </c>
+      <c r="B97" t="s">
+        <v>31</v>
+      </c>
+      <c r="C97" t="s">
         <v>74</v>
       </c>
-      <c r="D96">
+      <c r="D97">
         <v>550</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>120</v>
-      </c>
-      <c r="B97" t="s">
-        <v>54</v>
-      </c>
-      <c r="C97" t="s">
-        <v>70</v>
-      </c>
-      <c r="D97">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4">
       <c r="A98" t="s">
         <v>120</v>
       </c>
       <c r="B98" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C98" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D98">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4">
       <c r="A99" t="s">
         <v>120</v>
       </c>
@@ -2221,13 +2224,13 @@
         <v>30</v>
       </c>
       <c r="C99" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D99">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4">
       <c r="A100" t="s">
         <v>120</v>
       </c>
@@ -2235,23 +2238,37 @@
         <v>30</v>
       </c>
       <c r="C100" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D100">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4">
       <c r="A101" t="s">
         <v>120</v>
       </c>
       <c r="B101" t="s">
+        <v>30</v>
+      </c>
+      <c r="C101" t="s">
+        <v>75</v>
+      </c>
+      <c r="D101">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4">
+      <c r="A102" t="s">
+        <v>120</v>
+      </c>
+      <c r="B102" t="s">
         <v>45</v>
       </c>
-      <c r="C101" t="s">
+      <c r="C102" t="s">
         <v>76</v>
       </c>
-      <c r="D101">
+      <c r="D102">
         <v>450</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ExcelAdd: Adding one more row
</commit_message>
<xml_diff>
--- a/backend/data/cennik.xlsx
+++ b/backend/data/cennik.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\StronaMonika\backend\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\StronaMonikaSkonczona\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{455FFD8A-A8C2-4BB6-8C7C-23AFB0ABF20D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C91E4D42-CE74-43C1-A2A7-C04B984716D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="10356" xr2:uid="{4DB6F867-2552-414A-BFD2-AB60479A5D88}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="145">
   <si>
     <t>OPIS</t>
   </si>
@@ -462,13 +462,22 @@
   </si>
   <si>
     <t>Depilacja klatki piersiowej</t>
+  </si>
+  <si>
+    <t>+ 15min</t>
+  </si>
+  <si>
+    <t>Dodatkowa ampułka nanoigieł</t>
+  </si>
+  <si>
+    <t>+ 150</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -835,16 +844,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED3D7DE2-9127-49D9-96AA-B2504799E15F}">
-  <dimension ref="A1:D102"/>
-  <sheetFormatPr defaultColWidth="32" defaultRowHeight="14.25"/>
+  <dimension ref="A1:D103"/>
+  <sheetFormatPr defaultColWidth="32" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="39.125" customWidth="1"/>
-    <col min="2" max="2" width="17.75" customWidth="1"/>
-    <col min="3" max="3" width="49.375" customWidth="1"/>
-    <col min="4" max="4" width="18.125" customWidth="1"/>
+    <col min="1" max="1" width="39.109375" customWidth="1"/>
+    <col min="2" max="2" width="17.77734375" customWidth="1"/>
+    <col min="3" max="3" width="49.33203125" customWidth="1"/>
+    <col min="4" max="4" width="18.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -858,7 +867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -872,7 +881,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -886,7 +895,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -900,7 +909,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -914,7 +923,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -928,7 +937,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -942,7 +951,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -956,7 +965,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -970,7 +979,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -984,7 +993,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -998,7 +1007,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -1012,7 +1021,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -1026,7 +1035,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -1040,7 +1049,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -1054,7 +1063,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -1068,7 +1077,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>5</v>
       </c>
@@ -1082,7 +1091,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -1096,7 +1105,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -1110,7 +1119,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>11</v>
       </c>
@@ -1124,7 +1133,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -1138,7 +1147,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -1152,7 +1161,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -1166,7 +1175,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -1180,7 +1189,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>17</v>
       </c>
@@ -1194,7 +1203,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>18</v>
       </c>
@@ -1208,7 +1217,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>18</v>
       </c>
@@ -1222,7 +1231,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>20</v>
       </c>
@@ -1236,7 +1245,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>20</v>
       </c>
@@ -1250,7 +1259,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>122</v>
       </c>
@@ -1264,7 +1273,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>122</v>
       </c>
@@ -1278,7 +1287,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>122</v>
       </c>
@@ -1292,7 +1301,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>122</v>
       </c>
@@ -1306,7 +1315,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>122</v>
       </c>
@@ -1320,7 +1329,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>82</v>
       </c>
@@ -1334,7 +1343,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>82</v>
       </c>
@@ -1348,7 +1357,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>82</v>
       </c>
@@ -1362,7 +1371,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>82</v>
       </c>
@@ -1376,7 +1385,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>82</v>
       </c>
@@ -1390,7 +1399,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>121</v>
       </c>
@@ -1404,7 +1413,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>121</v>
       </c>
@@ -1418,7 +1427,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>121</v>
       </c>
@@ -1432,7 +1441,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:4">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>121</v>
       </c>
@@ -1446,7 +1455,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>121</v>
       </c>
@@ -1460,7 +1469,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:4">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>121</v>
       </c>
@@ -1474,7 +1483,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="46" spans="1:4">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>121</v>
       </c>
@@ -1488,7 +1497,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="47" spans="1:4">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>121</v>
       </c>
@@ -1502,7 +1511,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="48" spans="1:4">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>121</v>
       </c>
@@ -1516,7 +1525,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="49" spans="1:4">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>43</v>
       </c>
@@ -1530,7 +1539,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>43</v>
       </c>
@@ -1544,7 +1553,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>43</v>
       </c>
@@ -1558,7 +1567,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>46</v>
       </c>
@@ -1572,7 +1581,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>47</v>
       </c>
@@ -1586,7 +1595,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="54" spans="1:4">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>47</v>
       </c>
@@ -1600,7 +1609,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>47</v>
       </c>
@@ -1614,7 +1623,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>47</v>
       </c>
@@ -1628,7 +1637,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="57" spans="1:4">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>47</v>
       </c>
@@ -1642,7 +1651,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="58" spans="1:4">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>47</v>
       </c>
@@ -1656,7 +1665,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="59" spans="1:4">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>108</v>
       </c>
@@ -1670,7 +1679,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="60" spans="1:4">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>108</v>
       </c>
@@ -1684,7 +1693,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="61" spans="1:4">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>108</v>
       </c>
@@ -1698,7 +1707,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="62" spans="1:4">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>108</v>
       </c>
@@ -1712,7 +1721,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="63" spans="1:4">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>108</v>
       </c>
@@ -1726,7 +1735,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="64" spans="1:4">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>105</v>
       </c>
@@ -1740,7 +1749,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="65" spans="1:4">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>105</v>
       </c>
@@ -1754,7 +1763,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="66" spans="1:4">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>105</v>
       </c>
@@ -1768,7 +1777,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="67" spans="1:4">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>105</v>
       </c>
@@ -1782,7 +1791,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="68" spans="1:4">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>116</v>
       </c>
@@ -1796,7 +1805,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="69" spans="1:4">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>116</v>
       </c>
@@ -1810,7 +1819,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="70" spans="1:4">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>116</v>
       </c>
@@ -1824,7 +1833,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="71" spans="1:4">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>53</v>
       </c>
@@ -1838,7 +1847,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="72" spans="1:4">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>53</v>
       </c>
@@ -1852,7 +1861,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="73" spans="1:4">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>53</v>
       </c>
@@ -1866,7 +1875,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="74" spans="1:4">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>53</v>
       </c>
@@ -1880,7 +1889,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="75" spans="1:4">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>53</v>
       </c>
@@ -1894,7 +1903,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="76" spans="1:4">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>117</v>
       </c>
@@ -1908,7 +1917,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="77" spans="1:4">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>117</v>
       </c>
@@ -1922,7 +1931,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="78" spans="1:4">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>117</v>
       </c>
@@ -1936,7 +1945,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="79" spans="1:4">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>117</v>
       </c>
@@ -1950,7 +1959,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="80" spans="1:4">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>63</v>
       </c>
@@ -1964,7 +1973,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="81" spans="1:4">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>63</v>
       </c>
@@ -1978,7 +1987,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="82" spans="1:4">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>63</v>
       </c>
@@ -1992,7 +2001,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="83" spans="1:4">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>63</v>
       </c>
@@ -2006,7 +2015,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="84" spans="1:4">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>63</v>
       </c>
@@ -2020,7 +2029,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="85" spans="1:4">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>63</v>
       </c>
@@ -2034,7 +2043,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="86" spans="1:4">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>63</v>
       </c>
@@ -2048,7 +2057,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="87" spans="1:4">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>63</v>
       </c>
@@ -2062,7 +2071,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="88" spans="1:4">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>63</v>
       </c>
@@ -2076,7 +2085,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="89" spans="1:4">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>68</v>
       </c>
@@ -2090,7 +2099,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="90" spans="1:4">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>68</v>
       </c>
@@ -2104,35 +2113,35 @@
         <v>450</v>
       </c>
     </row>
-    <row r="91" spans="1:4">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>118</v>
-      </c>
-      <c r="B91" t="s">
-        <v>29</v>
+        <v>68</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>142</v>
       </c>
       <c r="C91" t="s">
-        <v>70</v>
-      </c>
-      <c r="D91">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4">
+        <v>143</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>118</v>
       </c>
       <c r="B92" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="C92" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D92">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>118</v>
       </c>
@@ -2140,55 +2149,55 @@
         <v>54</v>
       </c>
       <c r="C93" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D93">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>118</v>
       </c>
       <c r="B94" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C94" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D94">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>118</v>
       </c>
       <c r="B95" t="s">
+        <v>30</v>
+      </c>
+      <c r="C95" t="s">
+        <v>73</v>
+      </c>
+      <c r="D95">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>118</v>
+      </c>
+      <c r="B96" t="s">
         <v>39</v>
       </c>
-      <c r="C95" t="s">
+      <c r="C96" t="s">
         <v>74</v>
       </c>
-      <c r="D95">
+      <c r="D96">
         <v>350</v>
       </c>
     </row>
-    <row r="96" spans="1:4">
-      <c r="A96" t="s">
-        <v>119</v>
-      </c>
-      <c r="B96" t="s">
-        <v>31</v>
-      </c>
-      <c r="C96" t="s">
-        <v>73</v>
-      </c>
-      <c r="D96">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>119</v>
       </c>
@@ -2196,41 +2205,41 @@
         <v>31</v>
       </c>
       <c r="C97" t="s">
+        <v>73</v>
+      </c>
+      <c r="D97">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>119</v>
+      </c>
+      <c r="B98" t="s">
+        <v>31</v>
+      </c>
+      <c r="C98" t="s">
         <v>74</v>
       </c>
-      <c r="D97">
+      <c r="D98">
         <v>550</v>
       </c>
     </row>
-    <row r="98" spans="1:4">
-      <c r="A98" t="s">
-        <v>120</v>
-      </c>
-      <c r="B98" t="s">
-        <v>54</v>
-      </c>
-      <c r="C98" t="s">
-        <v>70</v>
-      </c>
-      <c r="D98">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>120</v>
       </c>
       <c r="B99" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C99" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D99">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>120</v>
       </c>
@@ -2238,13 +2247,13 @@
         <v>30</v>
       </c>
       <c r="C100" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D100">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>120</v>
       </c>
@@ -2252,23 +2261,37 @@
         <v>30</v>
       </c>
       <c r="C101" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D101">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>120</v>
       </c>
       <c r="B102" t="s">
+        <v>30</v>
+      </c>
+      <c r="C102" t="s">
+        <v>75</v>
+      </c>
+      <c r="D102">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>120</v>
+      </c>
+      <c r="B103" t="s">
         <v>45</v>
       </c>
-      <c r="C102" t="s">
+      <c r="C103" t="s">
         <v>76</v>
       </c>
-      <c r="D102">
+      <c r="D103">
         <v>450</v>
       </c>
     </row>

</xml_diff>